<commit_message>
Save in Ukelele 3.6.1 Modify QW from @win to Ωω (with AltGr) Only for macOS
</commit_message>
<xml_diff>
--- a/Images/WhiskKBLayouts.xlsx
+++ b/Images/WhiskKBLayouts.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10517"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/2Data/GitHub/Whiskeroff/WhiskKBLayouts/Images/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF31338C-3816-884A-B0A0-B699687B3E5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15" yWindow="465" windowWidth="38400" windowHeight="16440"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EN&amp;RU by Whisk" sheetId="7" r:id="rId1"/>
@@ -14,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="142">
   <si>
     <t>&lt;</t>
   </si>
@@ -398,9 +404,6 @@
   </si>
   <si>
     <t>§</t>
-  </si>
-  <si>
-    <t>⊞</t>
   </si>
   <si>
     <t>alt</t>
@@ -488,11 +491,17 @@
   <si>
     <t xml:space="preserve"> ¬</t>
   </si>
+  <si>
+    <t>Ω</t>
+  </si>
+  <si>
+    <t>ω</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="12">
     <font>
       <sz val="11"/>
@@ -734,27 +743,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -765,7 +766,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -788,7 +789,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -805,7 +806,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -831,7 +832,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -849,62 +850,21 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -912,48 +872,84 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -969,9 +965,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Стандартная">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1009,7 +1005,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Стандартная">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1081,7 +1077,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Стандартная">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1254,409 +1250,347 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BG21"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <dimension ref="B1:BG21"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="1.140625" style="13" customWidth="1"/>
-    <col min="2" max="2" width="4" style="13" customWidth="1"/>
-    <col min="3" max="3" width="0.7109375" style="13" customWidth="1"/>
-    <col min="4" max="4" width="4" style="13" customWidth="1"/>
-    <col min="5" max="5" width="0.7109375" style="13" customWidth="1"/>
-    <col min="6" max="6" width="4" style="13" customWidth="1"/>
-    <col min="7" max="7" width="0.7109375" style="13" customWidth="1"/>
-    <col min="8" max="8" width="4" style="13" customWidth="1"/>
-    <col min="9" max="9" width="0.7109375" style="13" customWidth="1"/>
-    <col min="10" max="10" width="4" style="13" customWidth="1"/>
-    <col min="11" max="11" width="0.7109375" style="13" customWidth="1"/>
-    <col min="12" max="12" width="4" style="13" customWidth="1"/>
-    <col min="13" max="13" width="0.7109375" style="13" customWidth="1"/>
-    <col min="14" max="14" width="4" style="13" customWidth="1"/>
-    <col min="15" max="15" width="0.7109375" style="13" customWidth="1"/>
-    <col min="16" max="16" width="4" style="13" customWidth="1"/>
-    <col min="17" max="17" width="0.7109375" style="13" customWidth="1"/>
-    <col min="18" max="18" width="4" style="13" customWidth="1"/>
-    <col min="19" max="19" width="0.7109375" style="13" customWidth="1"/>
-    <col min="20" max="20" width="4" style="13" customWidth="1"/>
-    <col min="21" max="21" width="0.7109375" style="13" customWidth="1"/>
-    <col min="22" max="22" width="4" style="13" customWidth="1"/>
-    <col min="23" max="23" width="0.7109375" style="13" customWidth="1"/>
-    <col min="24" max="24" width="4" style="13" customWidth="1"/>
-    <col min="25" max="25" width="0.7109375" style="13" customWidth="1"/>
-    <col min="26" max="26" width="4" style="13" customWidth="1"/>
-    <col min="27" max="27" width="0.7109375" style="13" customWidth="1"/>
-    <col min="28" max="28" width="4" style="13" customWidth="1"/>
-    <col min="29" max="29" width="0.7109375" style="13" customWidth="1"/>
-    <col min="30" max="30" width="4" style="13" customWidth="1"/>
-    <col min="31" max="31" width="0.7109375" style="13" customWidth="1"/>
-    <col min="32" max="32" width="4" style="13" customWidth="1"/>
-    <col min="33" max="33" width="0.7109375" style="13" customWidth="1"/>
-    <col min="34" max="34" width="4" style="13" customWidth="1"/>
-    <col min="35" max="35" width="0.7109375" style="13" customWidth="1"/>
-    <col min="36" max="36" width="4" style="13" customWidth="1"/>
-    <col min="37" max="37" width="0.7109375" style="13" customWidth="1"/>
-    <col min="38" max="38" width="4" style="13" customWidth="1"/>
-    <col min="39" max="39" width="0.7109375" style="13" customWidth="1"/>
-    <col min="40" max="40" width="4" style="13" customWidth="1"/>
-    <col min="41" max="41" width="0.7109375" style="13" customWidth="1"/>
-    <col min="42" max="42" width="4" style="13" customWidth="1"/>
-    <col min="43" max="43" width="0.7109375" style="13" customWidth="1"/>
-    <col min="44" max="44" width="4" style="13" customWidth="1"/>
-    <col min="45" max="45" width="0.7109375" style="13" customWidth="1"/>
-    <col min="46" max="46" width="4" style="13" customWidth="1"/>
-    <col min="47" max="47" width="0.7109375" style="13" customWidth="1"/>
-    <col min="48" max="48" width="4" style="13" customWidth="1"/>
-    <col min="49" max="49" width="0.7109375" style="13" customWidth="1"/>
-    <col min="50" max="50" width="4" style="13" customWidth="1"/>
-    <col min="51" max="51" width="0.7109375" style="13" customWidth="1"/>
-    <col min="52" max="52" width="4" style="13" customWidth="1"/>
-    <col min="53" max="53" width="0.7109375" style="13" customWidth="1"/>
-    <col min="54" max="54" width="4" style="13" customWidth="1"/>
-    <col min="55" max="55" width="0.7109375" style="13" customWidth="1"/>
-    <col min="56" max="56" width="4" style="13" customWidth="1"/>
-    <col min="57" max="57" width="0.7109375" style="13" customWidth="1"/>
-    <col min="58" max="58" width="4" style="13" customWidth="1"/>
-    <col min="59" max="59" width="1.140625" style="13" customWidth="1"/>
-    <col min="60" max="16384" width="9.140625" style="13"/>
+    <col min="1" max="1" width="1.1640625" style="8" customWidth="1"/>
+    <col min="2" max="2" width="4" style="8" customWidth="1"/>
+    <col min="3" max="3" width="0.6640625" style="8" customWidth="1"/>
+    <col min="4" max="4" width="4" style="8" customWidth="1"/>
+    <col min="5" max="5" width="0.6640625" style="8" customWidth="1"/>
+    <col min="6" max="6" width="4" style="8" customWidth="1"/>
+    <col min="7" max="7" width="0.6640625" style="8" customWidth="1"/>
+    <col min="8" max="8" width="4" style="8" customWidth="1"/>
+    <col min="9" max="9" width="0.6640625" style="8" customWidth="1"/>
+    <col min="10" max="10" width="4" style="8" customWidth="1"/>
+    <col min="11" max="11" width="0.6640625" style="8" customWidth="1"/>
+    <col min="12" max="12" width="4" style="8" customWidth="1"/>
+    <col min="13" max="13" width="0.6640625" style="8" customWidth="1"/>
+    <col min="14" max="14" width="4" style="8" customWidth="1"/>
+    <col min="15" max="15" width="0.6640625" style="8" customWidth="1"/>
+    <col min="16" max="16" width="4" style="8" customWidth="1"/>
+    <col min="17" max="17" width="0.6640625" style="8" customWidth="1"/>
+    <col min="18" max="18" width="4" style="8" customWidth="1"/>
+    <col min="19" max="19" width="0.6640625" style="8" customWidth="1"/>
+    <col min="20" max="20" width="4" style="8" customWidth="1"/>
+    <col min="21" max="21" width="0.6640625" style="8" customWidth="1"/>
+    <col min="22" max="22" width="4" style="8" customWidth="1"/>
+    <col min="23" max="23" width="0.6640625" style="8" customWidth="1"/>
+    <col min="24" max="24" width="4" style="8" customWidth="1"/>
+    <col min="25" max="25" width="0.6640625" style="8" customWidth="1"/>
+    <col min="26" max="26" width="4" style="8" customWidth="1"/>
+    <col min="27" max="27" width="0.6640625" style="8" customWidth="1"/>
+    <col min="28" max="28" width="4" style="8" customWidth="1"/>
+    <col min="29" max="29" width="0.6640625" style="8" customWidth="1"/>
+    <col min="30" max="30" width="4" style="8" customWidth="1"/>
+    <col min="31" max="31" width="0.6640625" style="8" customWidth="1"/>
+    <col min="32" max="32" width="4" style="8" customWidth="1"/>
+    <col min="33" max="33" width="0.6640625" style="8" customWidth="1"/>
+    <col min="34" max="34" width="4" style="8" customWidth="1"/>
+    <col min="35" max="35" width="0.6640625" style="8" customWidth="1"/>
+    <col min="36" max="36" width="4" style="8" customWidth="1"/>
+    <col min="37" max="37" width="0.6640625" style="8" customWidth="1"/>
+    <col min="38" max="38" width="4" style="8" customWidth="1"/>
+    <col min="39" max="39" width="0.6640625" style="8" customWidth="1"/>
+    <col min="40" max="40" width="4" style="8" customWidth="1"/>
+    <col min="41" max="41" width="0.6640625" style="8" customWidth="1"/>
+    <col min="42" max="42" width="4" style="8" customWidth="1"/>
+    <col min="43" max="43" width="0.6640625" style="8" customWidth="1"/>
+    <col min="44" max="44" width="4" style="8" customWidth="1"/>
+    <col min="45" max="45" width="0.6640625" style="8" customWidth="1"/>
+    <col min="46" max="46" width="4" style="8" customWidth="1"/>
+    <col min="47" max="47" width="0.6640625" style="8" customWidth="1"/>
+    <col min="48" max="48" width="4" style="8" customWidth="1"/>
+    <col min="49" max="49" width="0.6640625" style="8" customWidth="1"/>
+    <col min="50" max="50" width="4" style="8" customWidth="1"/>
+    <col min="51" max="51" width="0.6640625" style="8" customWidth="1"/>
+    <col min="52" max="52" width="4" style="8" customWidth="1"/>
+    <col min="53" max="53" width="0.6640625" style="8" customWidth="1"/>
+    <col min="54" max="54" width="4" style="8" customWidth="1"/>
+    <col min="55" max="55" width="0.6640625" style="8" customWidth="1"/>
+    <col min="56" max="56" width="4" style="8" customWidth="1"/>
+    <col min="57" max="57" width="0.6640625" style="8" customWidth="1"/>
+    <col min="58" max="58" width="4" style="8" customWidth="1"/>
+    <col min="59" max="59" width="1.1640625" style="8" customWidth="1"/>
+    <col min="60" max="16384" width="9.1640625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:59" ht="4.5" customHeight="1" thickBot="1">
-      <c r="A1" s="12"/>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
-      <c r="P1" s="12"/>
-      <c r="Q1" s="12"/>
-      <c r="R1" s="12"/>
-      <c r="S1" s="12"/>
-      <c r="T1" s="12"/>
-      <c r="U1" s="12"/>
-      <c r="V1" s="12"/>
-      <c r="W1" s="12" t="s">
+    <row r="1" spans="2:59" ht="4.5" customHeight="1" thickBot="1">
+      <c r="W1" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="X1" s="12"/>
-      <c r="Y1" s="12"/>
-      <c r="Z1" s="12"/>
-      <c r="AA1" s="12"/>
-      <c r="AB1" s="12"/>
-      <c r="AC1" s="12"/>
-      <c r="AD1" s="12"/>
-      <c r="AE1" s="12"/>
-      <c r="AF1" s="12"/>
-      <c r="AG1" s="12"/>
-      <c r="AH1" s="12"/>
-      <c r="AI1" s="12"/>
-      <c r="AJ1" s="12"/>
-      <c r="AK1" s="12"/>
-      <c r="AL1" s="12"/>
-      <c r="AM1" s="12"/>
-      <c r="AN1" s="12"/>
-      <c r="AO1" s="12"/>
-      <c r="AP1" s="12"/>
-      <c r="AQ1" s="12"/>
-      <c r="AR1" s="12"/>
-      <c r="AS1" s="12"/>
-      <c r="AT1" s="12"/>
-      <c r="AU1" s="12"/>
-      <c r="AV1" s="12"/>
-      <c r="AW1" s="12"/>
-      <c r="AX1" s="12"/>
-      <c r="AY1" s="12"/>
-      <c r="AZ1" s="12"/>
-      <c r="BA1" s="12"/>
-      <c r="BB1" s="12"/>
-      <c r="BC1" s="12"/>
-      <c r="BD1" s="12"/>
-      <c r="BE1" s="12"/>
-      <c r="BF1" s="12"/>
-      <c r="BG1" s="12"/>
     </row>
-    <row r="2" spans="1:59" ht="20.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="16" t="s">
+    <row r="2" spans="2:59" ht="21">
+      <c r="B2" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="17"/>
-      <c r="D2" s="18" t="s">
+      <c r="C2" s="11"/>
+      <c r="D2" s="12" t="s">
         <v>109</v>
       </c>
       <c r="E2" s="1"/>
-      <c r="F2" s="27" t="s">
+      <c r="F2" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="28"/>
-      <c r="H2" s="29" t="s">
+      <c r="G2" s="22"/>
+      <c r="H2" s="23" t="s">
         <v>18</v>
       </c>
       <c r="I2" s="1"/>
-      <c r="J2" s="27" t="s">
+      <c r="J2" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="28"/>
-      <c r="L2" s="29" t="s">
+      <c r="K2" s="22"/>
+      <c r="L2" s="23" t="s">
         <v>6</v>
       </c>
       <c r="M2" s="1"/>
-      <c r="N2" s="27" t="s">
+      <c r="N2" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="O2" s="28"/>
-      <c r="P2" s="29" t="s">
+      <c r="O2" s="22"/>
+      <c r="P2" s="23" t="s">
         <v>1</v>
       </c>
       <c r="Q2" s="1"/>
-      <c r="R2" s="27" t="s">
+      <c r="R2" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="S2" s="28"/>
-      <c r="T2" s="29" t="s">
+      <c r="S2" s="22"/>
+      <c r="T2" s="23" t="s">
         <v>19</v>
       </c>
       <c r="U2" s="1"/>
-      <c r="V2" s="27" t="s">
+      <c r="V2" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="W2" s="28"/>
-      <c r="X2" s="29" t="s">
+      <c r="W2" s="22"/>
+      <c r="X2" s="23" t="s">
         <v>97</v>
       </c>
       <c r="Y2" s="1"/>
-      <c r="Z2" s="27" t="s">
+      <c r="Z2" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="AA2" s="28"/>
-      <c r="AB2" s="29" t="s">
+      <c r="AA2" s="22"/>
+      <c r="AB2" s="23" t="s">
         <v>9</v>
       </c>
       <c r="AC2" s="1"/>
-      <c r="AD2" s="27" t="s">
+      <c r="AD2" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="AE2" s="28"/>
-      <c r="AF2" s="29" t="s">
+      <c r="AE2" s="22"/>
+      <c r="AF2" s="23" t="s">
         <v>2</v>
       </c>
       <c r="AG2" s="1"/>
-      <c r="AH2" s="27" t="s">
+      <c r="AH2" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="AI2" s="28"/>
-      <c r="AJ2" s="29" t="s">
+      <c r="AI2" s="22"/>
+      <c r="AJ2" s="23" t="s">
         <v>114</v>
       </c>
       <c r="AK2" s="1"/>
-      <c r="AL2" s="27" t="s">
+      <c r="AL2" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="AM2" s="28"/>
-      <c r="AN2" s="29" t="s">
+      <c r="AM2" s="22"/>
+      <c r="AN2" s="23" t="s">
         <v>4</v>
       </c>
       <c r="AO2" s="1"/>
-      <c r="AP2" s="27" t="s">
+      <c r="AP2" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="AQ2" s="28"/>
-      <c r="AR2" s="29" t="s">
+      <c r="AQ2" s="22"/>
+      <c r="AR2" s="23" t="s">
         <v>8</v>
       </c>
       <c r="AS2" s="1"/>
-      <c r="AT2" s="27" t="s">
+      <c r="AT2" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="AU2" s="28"/>
-      <c r="AV2" s="29" t="s">
+      <c r="AU2" s="22"/>
+      <c r="AV2" s="23" t="s">
         <v>117</v>
       </c>
       <c r="AW2" s="1"/>
-      <c r="AX2" s="27" t="s">
+      <c r="AX2" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="AY2" s="28"/>
-      <c r="AZ2" s="29" t="s">
+      <c r="AY2" s="22"/>
+      <c r="AZ2" s="23" t="s">
         <v>40</v>
       </c>
       <c r="BA2" s="1"/>
-      <c r="BB2" s="37"/>
-      <c r="BC2" s="38"/>
-      <c r="BD2" s="82" t="s">
+      <c r="BB2" s="31"/>
+      <c r="BC2" s="32"/>
+      <c r="BD2" s="60" t="s">
         <v>112</v>
       </c>
-      <c r="BE2" s="38"/>
-      <c r="BF2" s="44"/>
-      <c r="BG2" s="83"/>
+      <c r="BE2" s="32"/>
+      <c r="BF2" s="38"/>
+      <c r="BG2" s="55"/>
     </row>
-    <row r="3" spans="1:59" ht="7.5" customHeight="1">
-      <c r="A3" s="12"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="21"/>
+    <row r="3" spans="2:59" ht="7.5" customHeight="1">
+      <c r="B3" s="13"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="15"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="32"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="26"/>
       <c r="I3" s="1"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="31"/>
-      <c r="L3" s="32"/>
+      <c r="J3" s="24"/>
+      <c r="K3" s="25"/>
+      <c r="L3" s="26"/>
       <c r="M3" s="1"/>
-      <c r="N3" s="30"/>
-      <c r="O3" s="31"/>
-      <c r="P3" s="32"/>
+      <c r="N3" s="24"/>
+      <c r="O3" s="25"/>
+      <c r="P3" s="26"/>
       <c r="Q3" s="1"/>
-      <c r="R3" s="30"/>
-      <c r="S3" s="31"/>
-      <c r="T3" s="32"/>
+      <c r="R3" s="24"/>
+      <c r="S3" s="25"/>
+      <c r="T3" s="26"/>
       <c r="U3" s="1"/>
-      <c r="V3" s="30"/>
-      <c r="W3" s="31"/>
-      <c r="X3" s="32"/>
+      <c r="V3" s="24"/>
+      <c r="W3" s="25"/>
+      <c r="X3" s="26"/>
       <c r="Y3" s="1"/>
-      <c r="Z3" s="30"/>
-      <c r="AA3" s="31"/>
-      <c r="AB3" s="32"/>
+      <c r="Z3" s="24"/>
+      <c r="AA3" s="25"/>
+      <c r="AB3" s="26"/>
       <c r="AC3" s="1"/>
-      <c r="AD3" s="30"/>
-      <c r="AE3" s="31"/>
-      <c r="AF3" s="32"/>
+      <c r="AD3" s="24"/>
+      <c r="AE3" s="25"/>
+      <c r="AF3" s="26"/>
       <c r="AG3" s="1"/>
-      <c r="AH3" s="30"/>
-      <c r="AI3" s="31"/>
-      <c r="AJ3" s="32"/>
+      <c r="AH3" s="24"/>
+      <c r="AI3" s="25"/>
+      <c r="AJ3" s="26"/>
       <c r="AK3" s="1"/>
-      <c r="AL3" s="30"/>
-      <c r="AM3" s="31"/>
-      <c r="AN3" s="32"/>
+      <c r="AL3" s="24"/>
+      <c r="AM3" s="25"/>
+      <c r="AN3" s="26"/>
       <c r="AO3" s="1"/>
-      <c r="AP3" s="30"/>
-      <c r="AQ3" s="31"/>
-      <c r="AR3" s="32"/>
+      <c r="AP3" s="24"/>
+      <c r="AQ3" s="25"/>
+      <c r="AR3" s="26"/>
       <c r="AS3" s="1"/>
-      <c r="AT3" s="30"/>
-      <c r="AU3" s="31"/>
-      <c r="AV3" s="32"/>
+      <c r="AT3" s="24"/>
+      <c r="AU3" s="25"/>
+      <c r="AV3" s="26"/>
       <c r="AW3" s="1"/>
-      <c r="AX3" s="30"/>
-      <c r="AY3" s="31"/>
-      <c r="AZ3" s="32"/>
+      <c r="AX3" s="24"/>
+      <c r="AY3" s="25"/>
+      <c r="AZ3" s="26"/>
       <c r="BA3" s="1"/>
-      <c r="BB3" s="39"/>
-      <c r="BC3" s="40"/>
-      <c r="BD3" s="40"/>
-      <c r="BE3" s="40"/>
-      <c r="BF3" s="40"/>
-      <c r="BG3" s="41"/>
+      <c r="BB3" s="33"/>
+      <c r="BC3" s="34"/>
+      <c r="BD3" s="34"/>
+      <c r="BE3" s="34"/>
+      <c r="BF3" s="34"/>
+      <c r="BG3" s="35"/>
     </row>
-    <row r="4" spans="1:59" ht="21" thickBot="1">
-      <c r="A4" s="12"/>
-      <c r="B4" s="22" t="s">
+    <row r="4" spans="2:59" ht="22" thickBot="1">
+      <c r="B4" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="C4" s="23"/>
-      <c r="D4" s="24" t="s">
+      <c r="C4" s="17"/>
+      <c r="D4" s="18" t="s">
         <v>111</v>
       </c>
       <c r="E4" s="1"/>
-      <c r="F4" s="33">
+      <c r="F4" s="27">
         <v>1</v>
       </c>
-      <c r="G4" s="34"/>
-      <c r="H4" s="35"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="29"/>
       <c r="I4" s="1"/>
-      <c r="J4" s="33">
+      <c r="J4" s="27">
         <v>2</v>
       </c>
-      <c r="K4" s="34"/>
-      <c r="L4" s="35"/>
+      <c r="K4" s="28"/>
+      <c r="L4" s="29"/>
       <c r="M4" s="1"/>
-      <c r="N4" s="33">
+      <c r="N4" s="27">
         <v>3</v>
       </c>
-      <c r="O4" s="34"/>
-      <c r="P4" s="36"/>
+      <c r="O4" s="28"/>
+      <c r="P4" s="30"/>
       <c r="Q4" s="1"/>
-      <c r="R4" s="33">
+      <c r="R4" s="27">
         <v>4</v>
       </c>
-      <c r="S4" s="34"/>
-      <c r="T4" s="35"/>
+      <c r="S4" s="28"/>
+      <c r="T4" s="29"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="33">
+      <c r="V4" s="27">
         <v>5</v>
       </c>
-      <c r="W4" s="34"/>
-      <c r="X4" s="35"/>
+      <c r="W4" s="28"/>
+      <c r="X4" s="29"/>
       <c r="Y4" s="1"/>
-      <c r="Z4" s="33">
+      <c r="Z4" s="27">
         <v>6</v>
       </c>
-      <c r="AA4" s="34"/>
-      <c r="AB4" s="35"/>
+      <c r="AA4" s="28"/>
+      <c r="AB4" s="29"/>
       <c r="AC4" s="1"/>
-      <c r="AD4" s="33">
+      <c r="AD4" s="27">
         <v>7</v>
       </c>
-      <c r="AE4" s="34">
+      <c r="AE4" s="28">
         <v>7</v>
       </c>
-      <c r="AF4" s="35"/>
+      <c r="AF4" s="29"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="33">
+      <c r="AH4" s="27">
         <v>8</v>
       </c>
-      <c r="AI4" s="34"/>
-      <c r="AJ4" s="35"/>
+      <c r="AI4" s="28"/>
+      <c r="AJ4" s="29"/>
       <c r="AK4" s="1"/>
-      <c r="AL4" s="33">
+      <c r="AL4" s="27">
         <v>9</v>
       </c>
-      <c r="AM4" s="34"/>
-      <c r="AN4" s="35"/>
+      <c r="AM4" s="28"/>
+      <c r="AN4" s="29"/>
       <c r="AO4" s="1"/>
-      <c r="AP4" s="33">
+      <c r="AP4" s="27">
         <v>0</v>
       </c>
-      <c r="AQ4" s="34"/>
-      <c r="AR4" s="36"/>
+      <c r="AQ4" s="28"/>
+      <c r="AR4" s="30"/>
       <c r="AS4" s="1"/>
-      <c r="AT4" s="33" t="s">
+      <c r="AT4" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="AU4" s="34"/>
-      <c r="AV4" s="36"/>
+      <c r="AU4" s="28"/>
+      <c r="AV4" s="30"/>
       <c r="AW4" s="1"/>
-      <c r="AX4" s="33" t="s">
+      <c r="AX4" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="AY4" s="34"/>
-      <c r="AZ4" s="36"/>
+      <c r="AY4" s="28"/>
+      <c r="AZ4" s="30"/>
       <c r="BA4" s="1"/>
-      <c r="BB4" s="42"/>
-      <c r="BC4" s="43"/>
-      <c r="BD4" s="46"/>
-      <c r="BE4" s="43"/>
-      <c r="BF4" s="46"/>
-      <c r="BG4" s="84"/>
+      <c r="BB4" s="36"/>
+      <c r="BC4" s="37"/>
+      <c r="BD4" s="40"/>
+      <c r="BE4" s="37"/>
+      <c r="BF4" s="40"/>
+      <c r="BG4" s="61"/>
     </row>
-    <row r="5" spans="1:59" ht="4.5" customHeight="1" thickBot="1">
-      <c r="A5" s="12"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
+    <row r="5" spans="2:59" ht="4.5" customHeight="1" thickBot="1">
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -1710,279 +1644,275 @@
       <c r="BB5" s="1"/>
       <c r="BC5" s="1"/>
       <c r="BD5" s="1"/>
-      <c r="BE5" s="4"/>
-      <c r="BF5" s="4"/>
-      <c r="BG5" s="4"/>
+      <c r="BE5" s="1"/>
+      <c r="BF5" s="1"/>
+      <c r="BG5" s="1"/>
     </row>
-    <row r="6" spans="1:59" ht="20.25">
-      <c r="A6" s="12"/>
-      <c r="B6" s="37"/>
-      <c r="C6" s="38"/>
-      <c r="D6" s="44" t="s">
+    <row r="6" spans="2:59" ht="21">
+      <c r="B6" s="31"/>
+      <c r="C6" s="32"/>
+      <c r="D6" s="38" t="s">
         <v>98</v>
       </c>
-      <c r="E6" s="38"/>
-      <c r="F6" s="45"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="39"/>
       <c r="G6" s="1"/>
-      <c r="H6" s="48" t="s">
+      <c r="H6" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="I6" s="49"/>
-      <c r="J6" s="50" t="s">
-        <v>6</v>
+      <c r="I6" s="43"/>
+      <c r="J6" s="44" t="s">
+        <v>140</v>
       </c>
       <c r="K6" s="1"/>
-      <c r="L6" s="48" t="s">
+      <c r="L6" s="42" t="s">
         <v>53</v>
       </c>
-      <c r="M6" s="49"/>
-      <c r="N6" s="50" t="s">
-        <v>128</v>
+      <c r="M6" s="43"/>
+      <c r="N6" s="44" t="s">
+        <v>141</v>
       </c>
       <c r="O6" s="1"/>
-      <c r="P6" s="48" t="s">
+      <c r="P6" s="42" t="s">
         <v>51</v>
       </c>
-      <c r="Q6" s="49"/>
-      <c r="R6" s="50" t="s">
+      <c r="Q6" s="43"/>
+      <c r="R6" s="44" t="s">
         <v>31</v>
       </c>
       <c r="S6" s="1"/>
-      <c r="T6" s="48" t="s">
+      <c r="T6" s="42" t="s">
         <v>50</v>
       </c>
-      <c r="U6" s="49"/>
-      <c r="V6" s="50" t="s">
+      <c r="U6" s="43"/>
+      <c r="V6" s="44" t="s">
         <v>106</v>
       </c>
       <c r="W6" s="1"/>
-      <c r="X6" s="48" t="s">
+      <c r="X6" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="Y6" s="49"/>
-      <c r="Z6" s="50" t="s">
+      <c r="Y6" s="43"/>
+      <c r="Z6" s="44" t="s">
         <v>107</v>
       </c>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="48" t="s">
+      <c r="AB6" s="42" t="s">
         <v>48</v>
       </c>
-      <c r="AC6" s="49"/>
-      <c r="AD6" s="50" t="s">
+      <c r="AC6" s="43"/>
+      <c r="AD6" s="44" t="s">
         <v>103</v>
       </c>
       <c r="AE6" s="1"/>
-      <c r="AF6" s="48" t="s">
+      <c r="AF6" s="42" t="s">
         <v>47</v>
       </c>
-      <c r="AG6" s="49"/>
-      <c r="AH6" s="50" t="s">
+      <c r="AG6" s="43"/>
+      <c r="AH6" s="44" t="s">
         <v>125</v>
       </c>
       <c r="AI6" s="1"/>
-      <c r="AJ6" s="48" t="s">
+      <c r="AJ6" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="AK6" s="49"/>
-      <c r="AL6" s="50" t="s">
+      <c r="AK6" s="43"/>
+      <c r="AL6" s="44" t="s">
         <v>46</v>
       </c>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="48" t="s">
+      <c r="AN6" s="42" t="s">
         <v>52</v>
       </c>
-      <c r="AO6" s="49"/>
-      <c r="AP6" s="50" t="s">
+      <c r="AO6" s="43"/>
+      <c r="AP6" s="44" t="s">
         <v>115</v>
       </c>
       <c r="AQ6" s="1"/>
-      <c r="AR6" s="48" t="s">
+      <c r="AR6" s="42" t="s">
         <v>45</v>
       </c>
-      <c r="AS6" s="49"/>
-      <c r="AT6" s="50" t="s">
+      <c r="AS6" s="43"/>
+      <c r="AT6" s="44" t="s">
         <v>104</v>
       </c>
       <c r="AU6" s="1"/>
-      <c r="AV6" s="16" t="s">
+      <c r="AV6" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="AW6" s="17"/>
-      <c r="AX6" s="18" t="s">
+      <c r="AW6" s="11"/>
+      <c r="AX6" s="12" t="s">
         <v>32</v>
       </c>
       <c r="AY6" s="1"/>
-      <c r="AZ6" s="16" t="s">
+      <c r="AZ6" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="BA6" s="17"/>
-      <c r="BB6" s="18" t="s">
+      <c r="BA6" s="11"/>
+      <c r="BB6" s="12" t="s">
         <v>33</v>
       </c>
       <c r="BC6" s="1"/>
-      <c r="BD6" s="37"/>
-      <c r="BE6" s="85" t="s">
+      <c r="BD6" s="31"/>
+      <c r="BE6" s="62" t="s">
         <v>30</v>
       </c>
-      <c r="BF6" s="44"/>
-      <c r="BG6" s="83"/>
+      <c r="BF6" s="38"/>
+      <c r="BG6" s="55"/>
     </row>
-    <row r="7" spans="1:59" ht="7.5" customHeight="1">
-      <c r="A7" s="12"/>
-      <c r="B7" s="39"/>
-      <c r="C7" s="40"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="41"/>
+    <row r="7" spans="2:59" ht="7.5" customHeight="1">
+      <c r="B7" s="33"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="35"/>
       <c r="G7" s="1"/>
-      <c r="H7" s="51"/>
-      <c r="I7" s="52"/>
-      <c r="J7" s="53"/>
+      <c r="H7" s="45"/>
+      <c r="I7" s="46"/>
+      <c r="J7" s="47"/>
       <c r="K7" s="1"/>
-      <c r="L7" s="51"/>
-      <c r="M7" s="52"/>
-      <c r="N7" s="53"/>
+      <c r="L7" s="45"/>
+      <c r="M7" s="46"/>
+      <c r="N7" s="47"/>
       <c r="O7" s="1"/>
-      <c r="P7" s="51"/>
-      <c r="Q7" s="52"/>
-      <c r="R7" s="53"/>
+      <c r="P7" s="45"/>
+      <c r="Q7" s="46"/>
+      <c r="R7" s="47"/>
       <c r="S7" s="1"/>
-      <c r="T7" s="51"/>
-      <c r="U7" s="52"/>
-      <c r="V7" s="53"/>
+      <c r="T7" s="45"/>
+      <c r="U7" s="46"/>
+      <c r="V7" s="47"/>
       <c r="W7" s="1"/>
-      <c r="X7" s="51"/>
-      <c r="Y7" s="52"/>
-      <c r="Z7" s="53"/>
+      <c r="X7" s="45"/>
+      <c r="Y7" s="46"/>
+      <c r="Z7" s="47"/>
       <c r="AA7" s="1"/>
-      <c r="AB7" s="51"/>
-      <c r="AC7" s="52"/>
-      <c r="AD7" s="53"/>
+      <c r="AB7" s="45"/>
+      <c r="AC7" s="46"/>
+      <c r="AD7" s="47"/>
       <c r="AE7" s="1"/>
-      <c r="AF7" s="51"/>
-      <c r="AG7" s="52"/>
-      <c r="AH7" s="53"/>
+      <c r="AF7" s="45"/>
+      <c r="AG7" s="46"/>
+      <c r="AH7" s="47"/>
       <c r="AI7" s="1"/>
-      <c r="AJ7" s="51"/>
-      <c r="AK7" s="52"/>
-      <c r="AL7" s="53"/>
+      <c r="AJ7" s="45"/>
+      <c r="AK7" s="46"/>
+      <c r="AL7" s="47"/>
       <c r="AM7" s="1"/>
-      <c r="AN7" s="51"/>
-      <c r="AO7" s="52"/>
-      <c r="AP7" s="53"/>
+      <c r="AN7" s="45"/>
+      <c r="AO7" s="46"/>
+      <c r="AP7" s="47"/>
       <c r="AQ7" s="1"/>
-      <c r="AR7" s="51"/>
-      <c r="AS7" s="52"/>
-      <c r="AT7" s="53"/>
+      <c r="AR7" s="45"/>
+      <c r="AS7" s="46"/>
+      <c r="AT7" s="47"/>
       <c r="AU7" s="1"/>
-      <c r="AV7" s="19"/>
-      <c r="AW7" s="20"/>
-      <c r="AX7" s="21"/>
+      <c r="AV7" s="13"/>
+      <c r="AW7" s="14"/>
+      <c r="AX7" s="15"/>
       <c r="AY7" s="1"/>
-      <c r="AZ7" s="19"/>
-      <c r="BA7" s="20"/>
-      <c r="BB7" s="21"/>
+      <c r="AZ7" s="13"/>
+      <c r="BA7" s="14"/>
+      <c r="BB7" s="15"/>
       <c r="BC7" s="1"/>
-      <c r="BD7" s="39"/>
-      <c r="BE7" s="40"/>
-      <c r="BF7" s="40"/>
-      <c r="BG7" s="41"/>
+      <c r="BD7" s="33"/>
+      <c r="BE7" s="34"/>
+      <c r="BF7" s="34"/>
+      <c r="BG7" s="35"/>
     </row>
-    <row r="8" spans="1:59" ht="21" thickBot="1">
-      <c r="A8" s="12"/>
-      <c r="B8" s="42"/>
-      <c r="C8" s="43"/>
-      <c r="D8" s="46" t="s">
+    <row r="8" spans="2:59" ht="22" thickBot="1">
+      <c r="B8" s="36"/>
+      <c r="C8" s="37"/>
+      <c r="D8" s="40" t="s">
         <v>116</v>
       </c>
-      <c r="E8" s="43"/>
-      <c r="F8" s="59"/>
+      <c r="E8" s="37"/>
+      <c r="F8" s="53"/>
       <c r="G8" s="1"/>
-      <c r="H8" s="54"/>
-      <c r="I8" s="55"/>
-      <c r="J8" s="56" t="s">
+      <c r="H8" s="48"/>
+      <c r="I8" s="49"/>
+      <c r="J8" s="50" t="s">
         <v>73</v>
       </c>
       <c r="K8" s="1"/>
-      <c r="L8" s="54"/>
-      <c r="M8" s="55"/>
-      <c r="N8" s="56" t="s">
+      <c r="L8" s="48"/>
+      <c r="M8" s="49"/>
+      <c r="N8" s="50" t="s">
         <v>72</v>
       </c>
       <c r="O8" s="1"/>
-      <c r="P8" s="54"/>
-      <c r="Q8" s="55"/>
-      <c r="R8" s="56" t="s">
+      <c r="P8" s="48"/>
+      <c r="Q8" s="49"/>
+      <c r="R8" s="50" t="s">
         <v>71</v>
       </c>
       <c r="S8" s="1"/>
-      <c r="T8" s="54"/>
-      <c r="U8" s="55"/>
-      <c r="V8" s="56" t="s">
+      <c r="T8" s="48"/>
+      <c r="U8" s="49"/>
+      <c r="V8" s="50" t="s">
         <v>70</v>
       </c>
       <c r="W8" s="1"/>
-      <c r="X8" s="54"/>
-      <c r="Y8" s="55"/>
-      <c r="Z8" s="56" t="s">
+      <c r="X8" s="48"/>
+      <c r="Y8" s="49"/>
+      <c r="Z8" s="50" t="s">
         <v>69</v>
       </c>
       <c r="AA8" s="1"/>
-      <c r="AB8" s="54"/>
-      <c r="AC8" s="55"/>
-      <c r="AD8" s="56" t="s">
+      <c r="AB8" s="48"/>
+      <c r="AC8" s="49"/>
+      <c r="AD8" s="50" t="s">
         <v>68</v>
       </c>
       <c r="AE8" s="1"/>
-      <c r="AF8" s="54"/>
-      <c r="AG8" s="55"/>
-      <c r="AH8" s="56" t="s">
+      <c r="AF8" s="48"/>
+      <c r="AG8" s="49"/>
+      <c r="AH8" s="50" t="s">
         <v>67</v>
       </c>
       <c r="AI8" s="1"/>
-      <c r="AJ8" s="54"/>
-      <c r="AK8" s="55"/>
-      <c r="AL8" s="56" t="s">
+      <c r="AJ8" s="48"/>
+      <c r="AK8" s="49"/>
+      <c r="AL8" s="50" t="s">
         <v>66</v>
       </c>
       <c r="AM8" s="1"/>
-      <c r="AN8" s="54"/>
-      <c r="AO8" s="55"/>
-      <c r="AP8" s="56" t="s">
+      <c r="AN8" s="48"/>
+      <c r="AO8" s="49"/>
+      <c r="AP8" s="50" t="s">
         <v>65</v>
       </c>
       <c r="AQ8" s="1"/>
-      <c r="AR8" s="54"/>
-      <c r="AS8" s="55"/>
-      <c r="AT8" s="56" t="s">
+      <c r="AR8" s="48"/>
+      <c r="AS8" s="49"/>
+      <c r="AT8" s="50" t="s">
         <v>64</v>
       </c>
       <c r="AU8" s="1"/>
-      <c r="AV8" s="22" t="s">
+      <c r="AV8" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="AW8" s="23"/>
-      <c r="AX8" s="24" t="s">
+      <c r="AW8" s="17"/>
+      <c r="AX8" s="18" t="s">
         <v>36</v>
       </c>
       <c r="AY8" s="1"/>
-      <c r="AZ8" s="22" t="s">
+      <c r="AZ8" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="BA8" s="23"/>
-      <c r="BB8" s="24" t="s">
+      <c r="BA8" s="17"/>
+      <c r="BB8" s="18" t="s">
         <v>37</v>
       </c>
       <c r="BC8" s="1"/>
-      <c r="BD8" s="86"/>
-      <c r="BE8" s="43"/>
-      <c r="BF8" s="87"/>
-      <c r="BG8" s="41"/>
+      <c r="BD8" s="63"/>
+      <c r="BE8" s="37"/>
+      <c r="BF8" s="64"/>
+      <c r="BG8" s="35"/>
     </row>
-    <row r="9" spans="1:59" ht="4.5" customHeight="1" thickBot="1">
-      <c r="A9" s="12"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
+    <row r="9" spans="2:59" ht="4.5" customHeight="1" thickBot="1">
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
@@ -2036,805 +1966,793 @@
       <c r="BB9" s="1"/>
       <c r="BC9" s="1"/>
       <c r="BD9" s="1"/>
-      <c r="BE9" s="4"/>
-      <c r="BF9" s="39"/>
-      <c r="BG9" s="41"/>
+      <c r="BE9" s="1"/>
+      <c r="BF9" s="33"/>
+      <c r="BG9" s="35"/>
     </row>
-    <row r="10" spans="1:59" ht="20.25">
-      <c r="A10" s="12"/>
-      <c r="B10" s="37"/>
-      <c r="C10" s="38"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="44" t="s">
+    <row r="10" spans="2:59" ht="21">
+      <c r="B10" s="31"/>
+      <c r="C10" s="32"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="F10" s="44"/>
-      <c r="G10" s="38"/>
-      <c r="H10" s="45"/>
+      <c r="F10" s="38"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="39"/>
       <c r="I10" s="1"/>
-      <c r="J10" s="48" t="s">
+      <c r="J10" s="42" t="s">
         <v>55</v>
       </c>
-      <c r="K10" s="49"/>
-      <c r="L10" s="50" t="s">
+      <c r="K10" s="43"/>
+      <c r="L10" s="44" t="s">
         <v>101</v>
       </c>
       <c r="M10" s="1"/>
-      <c r="N10" s="48" t="s">
+      <c r="N10" s="42" t="s">
         <v>56</v>
       </c>
-      <c r="O10" s="49"/>
-      <c r="P10" s="50" t="s">
+      <c r="O10" s="43"/>
+      <c r="P10" s="44" t="s">
         <v>127</v>
       </c>
       <c r="Q10" s="1"/>
-      <c r="R10" s="48" t="s">
+      <c r="R10" s="42" t="s">
         <v>57</v>
       </c>
-      <c r="S10" s="49"/>
-      <c r="T10" s="50" t="s">
+      <c r="S10" s="43"/>
+      <c r="T10" s="44" t="s">
         <v>19</v>
       </c>
       <c r="U10" s="1"/>
-      <c r="V10" s="48" t="s">
+      <c r="V10" s="42" t="s">
         <v>58</v>
       </c>
-      <c r="W10" s="49"/>
-      <c r="X10" s="50" t="s">
+      <c r="W10" s="43"/>
+      <c r="X10" s="44" t="s">
         <v>105</v>
       </c>
       <c r="Y10" s="1"/>
-      <c r="Z10" s="48" t="s">
+      <c r="Z10" s="42" t="s">
         <v>59</v>
       </c>
-      <c r="AA10" s="49"/>
-      <c r="AB10" s="50" t="s">
+      <c r="AA10" s="43"/>
+      <c r="AB10" s="44" t="s">
         <v>100</v>
       </c>
       <c r="AC10" s="1"/>
-      <c r="AD10" s="48" t="s">
+      <c r="AD10" s="42" t="s">
         <v>60</v>
       </c>
-      <c r="AE10" s="49"/>
-      <c r="AF10" s="50" t="s">
+      <c r="AE10" s="43"/>
+      <c r="AF10" s="44" t="s">
         <v>121</v>
       </c>
       <c r="AG10" s="1"/>
-      <c r="AH10" s="48" t="s">
+      <c r="AH10" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="AI10" s="49"/>
-      <c r="AJ10" s="50" t="s">
+      <c r="AI10" s="43"/>
+      <c r="AJ10" s="44" t="s">
         <v>122</v>
       </c>
       <c r="AK10" s="1"/>
-      <c r="AL10" s="48" t="s">
+      <c r="AL10" s="42" t="s">
         <v>62</v>
       </c>
-      <c r="AM10" s="49"/>
-      <c r="AN10" s="50" t="s">
+      <c r="AM10" s="43"/>
+      <c r="AN10" s="44" t="s">
         <v>124</v>
       </c>
-      <c r="AO10" s="5"/>
-      <c r="AP10" s="48" t="s">
+      <c r="AO10" s="4"/>
+      <c r="AP10" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="AQ10" s="49"/>
-      <c r="AR10" s="57" t="s">
+      <c r="AQ10" s="43"/>
+      <c r="AR10" s="51" t="s">
         <v>63</v>
       </c>
-      <c r="AS10" s="10"/>
-      <c r="AT10" s="16" t="s">
+      <c r="AS10" s="7"/>
+      <c r="AT10" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="AU10" s="17"/>
-      <c r="AV10" s="18" t="s">
+      <c r="AU10" s="11"/>
+      <c r="AV10" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="AW10" s="10"/>
-      <c r="AX10" s="16" t="s">
+      <c r="AW10" s="7"/>
+      <c r="AX10" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="AY10" s="17"/>
-      <c r="AZ10" s="25" t="s">
+      <c r="AY10" s="11"/>
+      <c r="AZ10" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="BA10" s="5"/>
-      <c r="BB10" s="27" t="s">
+      <c r="BA10" s="4"/>
+      <c r="BB10" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="BC10" s="28"/>
-      <c r="BD10" s="29" t="s">
+      <c r="BC10" s="22"/>
+      <c r="BD10" s="23" t="s">
         <v>14</v>
       </c>
       <c r="BE10" s="3"/>
-      <c r="BF10" s="88"/>
-      <c r="BG10" s="41"/>
+      <c r="BF10" s="65"/>
+      <c r="BG10" s="35"/>
     </row>
-    <row r="11" spans="1:59" ht="7.5" customHeight="1">
-      <c r="A11" s="12"/>
-      <c r="B11" s="39"/>
-      <c r="C11" s="40"/>
-      <c r="D11" s="40"/>
-      <c r="E11" s="40"/>
-      <c r="F11" s="40"/>
-      <c r="G11" s="40"/>
-      <c r="H11" s="41"/>
+    <row r="11" spans="2:59" ht="7.5" customHeight="1">
+      <c r="B11" s="33"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="34"/>
+      <c r="H11" s="35"/>
       <c r="I11" s="1"/>
-      <c r="J11" s="51"/>
-      <c r="K11" s="52"/>
-      <c r="L11" s="53"/>
+      <c r="J11" s="45"/>
+      <c r="K11" s="46"/>
+      <c r="L11" s="47"/>
       <c r="M11" s="1"/>
-      <c r="N11" s="51"/>
-      <c r="O11" s="52"/>
-      <c r="P11" s="53"/>
+      <c r="N11" s="45"/>
+      <c r="O11" s="46"/>
+      <c r="P11" s="47"/>
       <c r="Q11" s="1"/>
-      <c r="R11" s="51"/>
-      <c r="S11" s="52"/>
-      <c r="T11" s="53"/>
+      <c r="R11" s="45"/>
+      <c r="S11" s="46"/>
+      <c r="T11" s="47"/>
       <c r="U11" s="1"/>
-      <c r="V11" s="51"/>
-      <c r="W11" s="52"/>
-      <c r="X11" s="53"/>
+      <c r="V11" s="45"/>
+      <c r="W11" s="46"/>
+      <c r="X11" s="47"/>
       <c r="Y11" s="1"/>
-      <c r="Z11" s="51"/>
-      <c r="AA11" s="52"/>
-      <c r="AB11" s="53"/>
+      <c r="Z11" s="45"/>
+      <c r="AA11" s="46"/>
+      <c r="AB11" s="47"/>
       <c r="AC11" s="1"/>
-      <c r="AD11" s="51"/>
-      <c r="AE11" s="52"/>
-      <c r="AF11" s="53"/>
+      <c r="AD11" s="45"/>
+      <c r="AE11" s="46"/>
+      <c r="AF11" s="47"/>
       <c r="AG11" s="1"/>
-      <c r="AH11" s="51"/>
-      <c r="AI11" s="52"/>
-      <c r="AJ11" s="53"/>
+      <c r="AH11" s="45"/>
+      <c r="AI11" s="46"/>
+      <c r="AJ11" s="47"/>
       <c r="AK11" s="1"/>
-      <c r="AL11" s="51"/>
-      <c r="AM11" s="52"/>
-      <c r="AN11" s="53"/>
-      <c r="AO11" s="5"/>
-      <c r="AP11" s="51"/>
-      <c r="AQ11" s="52"/>
-      <c r="AR11" s="53"/>
-      <c r="AS11" s="10"/>
-      <c r="AT11" s="19"/>
-      <c r="AU11" s="20"/>
-      <c r="AV11" s="21"/>
-      <c r="AW11" s="10"/>
-      <c r="AX11" s="19"/>
-      <c r="AY11" s="20"/>
-      <c r="AZ11" s="21"/>
-      <c r="BA11" s="5"/>
-      <c r="BB11" s="30"/>
-      <c r="BC11" s="31"/>
-      <c r="BD11" s="32"/>
+      <c r="AL11" s="45"/>
+      <c r="AM11" s="46"/>
+      <c r="AN11" s="47"/>
+      <c r="AO11" s="4"/>
+      <c r="AP11" s="45"/>
+      <c r="AQ11" s="46"/>
+      <c r="AR11" s="47"/>
+      <c r="AS11" s="7"/>
+      <c r="AT11" s="13"/>
+      <c r="AU11" s="14"/>
+      <c r="AV11" s="15"/>
+      <c r="AW11" s="7"/>
+      <c r="AX11" s="13"/>
+      <c r="AY11" s="14"/>
+      <c r="AZ11" s="15"/>
+      <c r="BA11" s="4"/>
+      <c r="BB11" s="24"/>
+      <c r="BC11" s="25"/>
+      <c r="BD11" s="26"/>
       <c r="BE11" s="3"/>
-      <c r="BF11" s="39"/>
-      <c r="BG11" s="41"/>
+      <c r="BF11" s="33"/>
+      <c r="BG11" s="35"/>
     </row>
-    <row r="12" spans="1:59" ht="21" thickBot="1">
-      <c r="A12" s="12"/>
-      <c r="B12" s="42"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="46"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="46"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="59"/>
+    <row r="12" spans="2:59" ht="22" thickBot="1">
+      <c r="B12" s="36"/>
+      <c r="C12" s="37"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="37"/>
+      <c r="F12" s="40"/>
+      <c r="G12" s="37"/>
+      <c r="H12" s="53"/>
       <c r="I12" s="1"/>
-      <c r="J12" s="54"/>
-      <c r="K12" s="55"/>
-      <c r="L12" s="56" t="s">
+      <c r="J12" s="48"/>
+      <c r="K12" s="49"/>
+      <c r="L12" s="50" t="s">
         <v>74</v>
       </c>
       <c r="M12" s="1"/>
-      <c r="N12" s="54"/>
-      <c r="O12" s="55"/>
-      <c r="P12" s="56" t="s">
+      <c r="N12" s="48"/>
+      <c r="O12" s="49"/>
+      <c r="P12" s="50" t="s">
         <v>75</v>
       </c>
       <c r="Q12" s="1"/>
-      <c r="R12" s="54"/>
-      <c r="S12" s="55"/>
-      <c r="T12" s="56" t="s">
+      <c r="R12" s="48"/>
+      <c r="S12" s="49"/>
+      <c r="T12" s="50" t="s">
         <v>76</v>
       </c>
       <c r="U12" s="1"/>
-      <c r="V12" s="54"/>
-      <c r="W12" s="55"/>
-      <c r="X12" s="56" t="s">
+      <c r="V12" s="48"/>
+      <c r="W12" s="49"/>
+      <c r="X12" s="50" t="s">
         <v>77</v>
       </c>
       <c r="Y12" s="1"/>
-      <c r="Z12" s="54"/>
-      <c r="AA12" s="55"/>
-      <c r="AB12" s="56" t="s">
+      <c r="Z12" s="48"/>
+      <c r="AA12" s="49"/>
+      <c r="AB12" s="50" t="s">
         <v>78</v>
       </c>
       <c r="AC12" s="1"/>
-      <c r="AD12" s="54"/>
-      <c r="AE12" s="55"/>
-      <c r="AF12" s="56" t="s">
+      <c r="AD12" s="48"/>
+      <c r="AE12" s="49"/>
+      <c r="AF12" s="50" t="s">
         <v>79</v>
       </c>
       <c r="AG12" s="1"/>
-      <c r="AH12" s="54"/>
-      <c r="AI12" s="55"/>
-      <c r="AJ12" s="56" t="s">
+      <c r="AH12" s="48"/>
+      <c r="AI12" s="49"/>
+      <c r="AJ12" s="50" t="s">
         <v>80</v>
       </c>
       <c r="AK12" s="1"/>
-      <c r="AL12" s="54"/>
-      <c r="AM12" s="55"/>
-      <c r="AN12" s="56" t="s">
+      <c r="AL12" s="48"/>
+      <c r="AM12" s="49"/>
+      <c r="AN12" s="50" t="s">
         <v>81</v>
       </c>
       <c r="AO12" s="1"/>
-      <c r="AP12" s="54"/>
-      <c r="AQ12" s="55"/>
-      <c r="AR12" s="56" t="s">
+      <c r="AP12" s="48"/>
+      <c r="AQ12" s="49"/>
+      <c r="AR12" s="50" t="s">
         <v>82</v>
       </c>
-      <c r="AS12" s="10"/>
-      <c r="AT12" s="22" t="s">
+      <c r="AS12" s="7"/>
+      <c r="AT12" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="AU12" s="23"/>
-      <c r="AV12" s="24" t="s">
+      <c r="AU12" s="17"/>
+      <c r="AV12" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="AW12" s="10"/>
-      <c r="AX12" s="26" t="s">
+      <c r="AW12" s="7"/>
+      <c r="AX12" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="AY12" s="23"/>
-      <c r="AZ12" s="24" t="s">
+      <c r="AY12" s="17"/>
+      <c r="AZ12" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="BA12" s="5"/>
-      <c r="BB12" s="33" t="s">
+      <c r="BA12" s="4"/>
+      <c r="BB12" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="BC12" s="34"/>
-      <c r="BD12" s="35"/>
+      <c r="BC12" s="28"/>
+      <c r="BD12" s="29"/>
       <c r="BE12" s="3"/>
-      <c r="BF12" s="42"/>
-      <c r="BG12" s="84"/>
+      <c r="BF12" s="36"/>
+      <c r="BG12" s="61"/>
     </row>
-    <row r="13" spans="1:59" ht="4.5" customHeight="1" thickBot="1">
-      <c r="A13" s="12"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
+    <row r="13" spans="2:59" ht="4.5" customHeight="1" thickBot="1">
+      <c r="B13" s="5"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
       <c r="G13" s="1"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
       <c r="K13" s="1"/>
-      <c r="L13" s="8"/>
-      <c r="M13" s="8"/>
-      <c r="N13" s="8"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="5"/>
       <c r="O13" s="1"/>
-      <c r="P13" s="8"/>
-      <c r="Q13" s="8"/>
-      <c r="R13" s="8"/>
+      <c r="P13" s="5"/>
+      <c r="Q13" s="5"/>
+      <c r="R13" s="5"/>
       <c r="S13" s="1"/>
-      <c r="T13" s="8"/>
-      <c r="U13" s="8"/>
-      <c r="V13" s="8"/>
+      <c r="T13" s="5"/>
+      <c r="U13" s="5"/>
+      <c r="V13" s="5"/>
       <c r="W13" s="1"/>
-      <c r="X13" s="8"/>
-      <c r="Y13" s="8"/>
-      <c r="Z13" s="8"/>
+      <c r="X13" s="5"/>
+      <c r="Y13" s="5"/>
+      <c r="Z13" s="5"/>
       <c r="AA13" s="1"/>
-      <c r="AB13" s="8"/>
-      <c r="AC13" s="8"/>
-      <c r="AD13" s="8"/>
+      <c r="AB13" s="5"/>
+      <c r="AC13" s="5"/>
+      <c r="AD13" s="5"/>
       <c r="AE13" s="1"/>
-      <c r="AF13" s="8"/>
-      <c r="AG13" s="8"/>
-      <c r="AH13" s="8"/>
+      <c r="AF13" s="5"/>
+      <c r="AG13" s="5"/>
+      <c r="AH13" s="5"/>
       <c r="AI13" s="1"/>
-      <c r="AJ13" s="8"/>
-      <c r="AK13" s="8"/>
-      <c r="AL13" s="8"/>
+      <c r="AJ13" s="5"/>
+      <c r="AK13" s="5"/>
+      <c r="AL13" s="5"/>
       <c r="AM13" s="1"/>
-      <c r="AN13" s="8"/>
-      <c r="AO13" s="8"/>
-      <c r="AP13" s="8"/>
+      <c r="AN13" s="5"/>
+      <c r="AO13" s="5"/>
+      <c r="AP13" s="5"/>
       <c r="AQ13" s="1"/>
-      <c r="AR13" s="8"/>
-      <c r="AS13" s="8"/>
-      <c r="AT13" s="8"/>
+      <c r="AR13" s="5"/>
+      <c r="AS13" s="5"/>
+      <c r="AT13" s="5"/>
       <c r="AU13" s="1"/>
       <c r="AV13" s="2"/>
-      <c r="AW13" s="11"/>
-      <c r="AX13" s="11"/>
-      <c r="AY13" s="11"/>
+      <c r="AW13" s="1"/>
+      <c r="AX13" s="1"/>
+      <c r="AY13" s="1"/>
       <c r="AZ13" s="1"/>
       <c r="BA13" s="1"/>
       <c r="BB13" s="1"/>
       <c r="BC13" s="1"/>
       <c r="BD13" s="1"/>
-      <c r="BE13" s="4"/>
-      <c r="BF13" s="4"/>
-      <c r="BG13" s="4"/>
+      <c r="BE13" s="1"/>
+      <c r="BF13" s="1"/>
+      <c r="BG13" s="1"/>
     </row>
-    <row r="14" spans="1:59" ht="20.25">
-      <c r="A14" s="12"/>
-      <c r="B14" s="37"/>
-      <c r="C14" s="38"/>
-      <c r="D14" s="44" t="s">
+    <row r="14" spans="2:59" ht="21">
+      <c r="B14" s="31"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="E14" s="38"/>
-      <c r="F14" s="45"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="I14" s="38"/>
-      <c r="J14" s="45"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="48" t="s">
+      <c r="E14" s="32"/>
+      <c r="F14" s="39"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="I14" s="32"/>
+      <c r="J14" s="39"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="42" t="s">
         <v>83</v>
       </c>
-      <c r="M14" s="49"/>
-      <c r="N14" s="50" t="s">
+      <c r="M14" s="43"/>
+      <c r="N14" s="44" t="s">
         <v>126</v>
       </c>
-      <c r="O14" s="10"/>
-      <c r="P14" s="48" t="s">
+      <c r="O14" s="7"/>
+      <c r="P14" s="42" t="s">
         <v>84</v>
       </c>
-      <c r="Q14" s="49"/>
-      <c r="R14" s="50" t="s">
+      <c r="Q14" s="43"/>
+      <c r="R14" s="44" t="s">
         <v>84</v>
       </c>
-      <c r="S14" s="10"/>
-      <c r="T14" s="48" t="s">
+      <c r="S14" s="7"/>
+      <c r="T14" s="42" t="s">
         <v>85</v>
       </c>
-      <c r="U14" s="49"/>
-      <c r="V14" s="50" t="s">
+      <c r="U14" s="43"/>
+      <c r="V14" s="44" t="s">
         <v>108</v>
       </c>
-      <c r="W14" s="10"/>
-      <c r="X14" s="48" t="s">
+      <c r="W14" s="7"/>
+      <c r="X14" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="Y14" s="49"/>
-      <c r="Z14" s="50" t="s">
+      <c r="Y14" s="43"/>
+      <c r="Z14" s="44" t="s">
         <v>86</v>
       </c>
-      <c r="AA14" s="10"/>
-      <c r="AB14" s="48" t="s">
+      <c r="AA14" s="7"/>
+      <c r="AB14" s="42" t="s">
         <v>87</v>
       </c>
-      <c r="AC14" s="49"/>
-      <c r="AD14" s="50" t="s">
+      <c r="AC14" s="43"/>
+      <c r="AD14" s="44" t="s">
         <v>102</v>
       </c>
-      <c r="AE14" s="10"/>
-      <c r="AF14" s="48" t="s">
+      <c r="AE14" s="7"/>
+      <c r="AF14" s="42" t="s">
         <v>88</v>
       </c>
-      <c r="AG14" s="49"/>
-      <c r="AH14" s="50" t="s">
+      <c r="AG14" s="43"/>
+      <c r="AH14" s="44" t="s">
         <v>123</v>
       </c>
-      <c r="AI14" s="10"/>
-      <c r="AJ14" s="48" t="s">
+      <c r="AI14" s="7"/>
+      <c r="AJ14" s="42" t="s">
         <v>89</v>
       </c>
-      <c r="AK14" s="49"/>
-      <c r="AL14" s="58" t="s">
-        <v>131</v>
-      </c>
-      <c r="AM14" s="10"/>
-      <c r="AN14" s="16" t="s">
+      <c r="AK14" s="43"/>
+      <c r="AL14" s="52" t="s">
+        <v>130</v>
+      </c>
+      <c r="AM14" s="7"/>
+      <c r="AN14" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="AO14" s="17"/>
-      <c r="AP14" s="18" t="s">
+      <c r="AO14" s="11"/>
+      <c r="AP14" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="AQ14" s="10"/>
-      <c r="AR14" s="16" t="s">
+      <c r="AQ14" s="7"/>
+      <c r="AR14" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="AS14" s="17"/>
-      <c r="AT14" s="18" t="s">
+      <c r="AS14" s="11"/>
+      <c r="AT14" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="AU14" s="6"/>
-      <c r="AV14" s="27" t="s">
+      <c r="AU14" s="3"/>
+      <c r="AV14" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="AW14" s="28"/>
-      <c r="AX14" s="29" t="s">
+      <c r="AW14" s="22"/>
+      <c r="AX14" s="23" t="s">
         <v>110</v>
       </c>
-      <c r="AY14" s="11"/>
-      <c r="AZ14" s="37"/>
-      <c r="BA14" s="38"/>
-      <c r="BB14" s="38"/>
-      <c r="BC14" s="47" t="s">
+      <c r="AY14" s="1"/>
+      <c r="AZ14" s="31"/>
+      <c r="BA14" s="32"/>
+      <c r="BB14" s="32"/>
+      <c r="BC14" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="BD14" s="44"/>
-      <c r="BE14" s="38"/>
-      <c r="BF14" s="44"/>
-      <c r="BG14" s="83"/>
+      <c r="BD14" s="38"/>
+      <c r="BE14" s="32"/>
+      <c r="BF14" s="38"/>
+      <c r="BG14" s="55"/>
     </row>
-    <row r="15" spans="1:59" ht="7.5" customHeight="1">
-      <c r="A15" s="12"/>
-      <c r="B15" s="39"/>
-      <c r="C15" s="40"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="41"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="39"/>
-      <c r="I15" s="40"/>
-      <c r="J15" s="41"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="51"/>
-      <c r="M15" s="52"/>
-      <c r="N15" s="53"/>
-      <c r="O15" s="10"/>
-      <c r="P15" s="51"/>
-      <c r="Q15" s="52"/>
-      <c r="R15" s="53"/>
-      <c r="S15" s="10"/>
-      <c r="T15" s="51"/>
-      <c r="U15" s="52"/>
-      <c r="V15" s="53"/>
-      <c r="W15" s="10"/>
-      <c r="X15" s="51"/>
-      <c r="Y15" s="52"/>
-      <c r="Z15" s="53"/>
-      <c r="AA15" s="10"/>
-      <c r="AB15" s="51"/>
-      <c r="AC15" s="52"/>
-      <c r="AD15" s="53"/>
-      <c r="AE15" s="10"/>
-      <c r="AF15" s="51"/>
-      <c r="AG15" s="52"/>
-      <c r="AH15" s="53"/>
-      <c r="AI15" s="10"/>
-      <c r="AJ15" s="51"/>
-      <c r="AK15" s="52"/>
-      <c r="AL15" s="53"/>
-      <c r="AM15" s="10"/>
-      <c r="AN15" s="19"/>
-      <c r="AO15" s="20"/>
-      <c r="AP15" s="21"/>
-      <c r="AQ15" s="10"/>
-      <c r="AR15" s="19"/>
-      <c r="AS15" s="20"/>
-      <c r="AT15" s="21"/>
-      <c r="AU15" s="6"/>
-      <c r="AV15" s="30"/>
-      <c r="AW15" s="31"/>
-      <c r="AX15" s="32"/>
-      <c r="AY15" s="11"/>
-      <c r="AZ15" s="39"/>
-      <c r="BA15" s="40"/>
-      <c r="BB15" s="40"/>
-      <c r="BC15" s="40"/>
-      <c r="BD15" s="40"/>
-      <c r="BE15" s="40"/>
-      <c r="BF15" s="40"/>
-      <c r="BG15" s="41"/>
+    <row r="15" spans="2:59" ht="7.5" customHeight="1">
+      <c r="B15" s="33"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="35"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="33"/>
+      <c r="I15" s="34"/>
+      <c r="J15" s="35"/>
+      <c r="K15" s="7"/>
+      <c r="L15" s="45"/>
+      <c r="M15" s="46"/>
+      <c r="N15" s="47"/>
+      <c r="O15" s="7"/>
+      <c r="P15" s="45"/>
+      <c r="Q15" s="46"/>
+      <c r="R15" s="47"/>
+      <c r="S15" s="7"/>
+      <c r="T15" s="45"/>
+      <c r="U15" s="46"/>
+      <c r="V15" s="47"/>
+      <c r="W15" s="7"/>
+      <c r="X15" s="45"/>
+      <c r="Y15" s="46"/>
+      <c r="Z15" s="47"/>
+      <c r="AA15" s="7"/>
+      <c r="AB15" s="45"/>
+      <c r="AC15" s="46"/>
+      <c r="AD15" s="47"/>
+      <c r="AE15" s="7"/>
+      <c r="AF15" s="45"/>
+      <c r="AG15" s="46"/>
+      <c r="AH15" s="47"/>
+      <c r="AI15" s="7"/>
+      <c r="AJ15" s="45"/>
+      <c r="AK15" s="46"/>
+      <c r="AL15" s="47"/>
+      <c r="AM15" s="7"/>
+      <c r="AN15" s="13"/>
+      <c r="AO15" s="14"/>
+      <c r="AP15" s="15"/>
+      <c r="AQ15" s="7"/>
+      <c r="AR15" s="13"/>
+      <c r="AS15" s="14"/>
+      <c r="AT15" s="15"/>
+      <c r="AU15" s="3"/>
+      <c r="AV15" s="24"/>
+      <c r="AW15" s="25"/>
+      <c r="AX15" s="26"/>
+      <c r="AY15" s="1"/>
+      <c r="AZ15" s="33"/>
+      <c r="BA15" s="34"/>
+      <c r="BB15" s="34"/>
+      <c r="BC15" s="34"/>
+      <c r="BD15" s="34"/>
+      <c r="BE15" s="34"/>
+      <c r="BF15" s="34"/>
+      <c r="BG15" s="35"/>
     </row>
-    <row r="16" spans="1:59" ht="21" thickBot="1">
-      <c r="A16" s="12"/>
-      <c r="B16" s="42"/>
-      <c r="C16" s="43"/>
-      <c r="D16" s="46"/>
-      <c r="E16" s="43"/>
-      <c r="F16" s="59"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="42" t="s">
-        <v>6</v>
-      </c>
-      <c r="I16" s="43"/>
-      <c r="J16" s="59"/>
-      <c r="K16" s="10"/>
-      <c r="L16" s="54"/>
-      <c r="M16" s="55"/>
-      <c r="N16" s="56" t="s">
+    <row r="16" spans="2:59" ht="22" thickBot="1">
+      <c r="B16" s="36"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="37"/>
+      <c r="F16" s="53"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="36"/>
+      <c r="I16" s="37"/>
+      <c r="J16" s="53"/>
+      <c r="K16" s="7"/>
+      <c r="L16" s="48"/>
+      <c r="M16" s="49"/>
+      <c r="N16" s="50" t="s">
         <v>96</v>
       </c>
       <c r="O16" s="1"/>
-      <c r="P16" s="54"/>
-      <c r="Q16" s="55"/>
-      <c r="R16" s="56" t="s">
+      <c r="P16" s="48"/>
+      <c r="Q16" s="49"/>
+      <c r="R16" s="50" t="s">
         <v>95</v>
       </c>
       <c r="S16" s="1"/>
-      <c r="T16" s="54"/>
-      <c r="U16" s="55"/>
-      <c r="V16" s="56" t="s">
+      <c r="T16" s="48"/>
+      <c r="U16" s="49"/>
+      <c r="V16" s="50" t="s">
         <v>94</v>
       </c>
       <c r="W16" s="1"/>
-      <c r="X16" s="54"/>
-      <c r="Y16" s="55"/>
-      <c r="Z16" s="56" t="s">
+      <c r="X16" s="48"/>
+      <c r="Y16" s="49"/>
+      <c r="Z16" s="50" t="s">
         <v>93</v>
       </c>
       <c r="AA16" s="1"/>
-      <c r="AB16" s="54"/>
-      <c r="AC16" s="55"/>
-      <c r="AD16" s="56" t="s">
+      <c r="AB16" s="48"/>
+      <c r="AC16" s="49"/>
+      <c r="AD16" s="50" t="s">
         <v>92</v>
       </c>
       <c r="AE16" s="1"/>
-      <c r="AF16" s="54"/>
-      <c r="AG16" s="55"/>
-      <c r="AH16" s="56" t="s">
+      <c r="AF16" s="48"/>
+      <c r="AG16" s="49"/>
+      <c r="AH16" s="50" t="s">
         <v>91</v>
       </c>
       <c r="AI16" s="1"/>
-      <c r="AJ16" s="54"/>
-      <c r="AK16" s="55"/>
-      <c r="AL16" s="56" t="s">
+      <c r="AJ16" s="48"/>
+      <c r="AK16" s="49"/>
+      <c r="AL16" s="50" t="s">
         <v>90</v>
       </c>
-      <c r="AM16" s="10"/>
-      <c r="AN16" s="22" t="s">
+      <c r="AM16" s="7"/>
+      <c r="AN16" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="AO16" s="23"/>
-      <c r="AP16" s="24" t="s">
+      <c r="AO16" s="17"/>
+      <c r="AP16" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="AQ16" s="10"/>
-      <c r="AR16" s="22" t="s">
+      <c r="AQ16" s="7"/>
+      <c r="AR16" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="AS16" s="23"/>
-      <c r="AT16" s="24" t="s">
+      <c r="AS16" s="17"/>
+      <c r="AT16" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="AU16" s="6"/>
-      <c r="AV16" s="33" t="s">
+      <c r="AU16" s="3"/>
+      <c r="AV16" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="AW16" s="34"/>
-      <c r="AX16" s="35"/>
-      <c r="AY16" s="11"/>
-      <c r="AZ16" s="42"/>
-      <c r="BA16" s="43"/>
-      <c r="BB16" s="46"/>
-      <c r="BC16" s="43"/>
-      <c r="BD16" s="46"/>
-      <c r="BE16" s="43"/>
-      <c r="BF16" s="46"/>
-      <c r="BG16" s="84"/>
+      <c r="AW16" s="28"/>
+      <c r="AX16" s="29"/>
+      <c r="AY16" s="1"/>
+      <c r="AZ16" s="36"/>
+      <c r="BA16" s="37"/>
+      <c r="BB16" s="40"/>
+      <c r="BC16" s="37"/>
+      <c r="BD16" s="40"/>
+      <c r="BE16" s="37"/>
+      <c r="BF16" s="40"/>
+      <c r="BG16" s="61"/>
     </row>
-    <row r="17" spans="1:59" ht="4.5" customHeight="1" thickBot="1"/>
-    <row r="18" spans="1:59" ht="21" customHeight="1" thickBot="1">
-      <c r="A18" s="12"/>
-      <c r="B18" s="60" t="s">
+    <row r="17" spans="2:59" ht="4.5" customHeight="1" thickBot="1"/>
+    <row r="18" spans="2:59" ht="21" customHeight="1" thickBot="1">
+      <c r="B18" s="70" t="s">
+        <v>132</v>
+      </c>
+      <c r="C18" s="71"/>
+      <c r="D18" s="72"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="54"/>
+      <c r="G18" s="32"/>
+      <c r="H18" s="55"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="67" t="s">
         <v>133</v>
       </c>
-      <c r="C18" s="61"/>
-      <c r="D18" s="62"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="69"/>
-      <c r="G18" s="70"/>
-      <c r="H18" s="71"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="72" t="s">
+      <c r="K18" s="68"/>
+      <c r="L18" s="69"/>
+      <c r="N18" s="70" t="s">
         <v>134</v>
       </c>
-      <c r="K18" s="73"/>
-      <c r="L18" s="74"/>
-      <c r="N18" s="60" t="s">
+      <c r="O18" s="71"/>
+      <c r="P18" s="71"/>
+      <c r="Q18" s="71"/>
+      <c r="R18" s="72"/>
+      <c r="S18" s="1"/>
+      <c r="T18" s="79" t="s">
+        <v>136</v>
+      </c>
+      <c r="U18" s="80"/>
+      <c r="V18" s="80"/>
+      <c r="W18" s="80"/>
+      <c r="X18" s="80"/>
+      <c r="Y18" s="80"/>
+      <c r="Z18" s="80"/>
+      <c r="AA18" s="80"/>
+      <c r="AB18" s="80"/>
+      <c r="AC18" s="80"/>
+      <c r="AD18" s="80"/>
+      <c r="AE18" s="80"/>
+      <c r="AF18" s="80"/>
+      <c r="AG18" s="80"/>
+      <c r="AH18" s="80"/>
+      <c r="AI18" s="80"/>
+      <c r="AJ18" s="80"/>
+      <c r="AK18" s="80"/>
+      <c r="AL18" s="81"/>
+      <c r="AM18" s="1"/>
+      <c r="AN18" s="88" t="s">
         <v>135</v>
       </c>
-      <c r="O18" s="61"/>
-      <c r="P18" s="61"/>
-      <c r="Q18" s="61"/>
-      <c r="R18" s="62"/>
-      <c r="S18" s="1"/>
-      <c r="T18" s="91" t="s">
+      <c r="AO18" s="71"/>
+      <c r="AP18" s="72"/>
+      <c r="AQ18" s="1"/>
+      <c r="AR18" s="67" t="s">
+        <v>133</v>
+      </c>
+      <c r="AS18" s="68"/>
+      <c r="AT18" s="69"/>
+      <c r="AU18" s="1"/>
+      <c r="AV18" s="70" t="s">
+        <v>132</v>
+      </c>
+      <c r="AW18" s="71"/>
+      <c r="AX18" s="72"/>
+      <c r="AY18" s="1"/>
+      <c r="AZ18" s="6"/>
+      <c r="BA18" s="1"/>
+      <c r="BB18" s="66" t="s">
         <v>137</v>
       </c>
-      <c r="U18" s="92"/>
-      <c r="V18" s="92"/>
-      <c r="W18" s="92"/>
-      <c r="X18" s="92"/>
-      <c r="Y18" s="92"/>
-      <c r="Z18" s="92"/>
-      <c r="AA18" s="92"/>
-      <c r="AB18" s="92"/>
-      <c r="AC18" s="92"/>
-      <c r="AD18" s="92"/>
-      <c r="AE18" s="92"/>
-      <c r="AF18" s="92"/>
-      <c r="AG18" s="92"/>
-      <c r="AH18" s="92"/>
-      <c r="AI18" s="92"/>
-      <c r="AJ18" s="92"/>
-      <c r="AK18" s="92"/>
-      <c r="AL18" s="93"/>
-      <c r="AM18" s="1"/>
-      <c r="AN18" s="90" t="s">
-        <v>136</v>
-      </c>
-      <c r="AO18" s="61"/>
-      <c r="AP18" s="62"/>
-      <c r="AQ18" s="1"/>
-      <c r="AR18" s="72" t="s">
-        <v>134</v>
-      </c>
-      <c r="AS18" s="73"/>
-      <c r="AT18" s="74"/>
-      <c r="AU18" s="1"/>
-      <c r="AV18" s="60" t="s">
-        <v>133</v>
-      </c>
-      <c r="AW18" s="61"/>
-      <c r="AX18" s="62"/>
-      <c r="AY18" s="1"/>
-      <c r="AZ18" s="14"/>
-      <c r="BA18" s="1"/>
-      <c r="BB18" s="89" t="s">
-        <v>138</v>
-      </c>
-      <c r="BC18" s="15"/>
-      <c r="BD18" s="14"/>
-      <c r="BE18" s="4"/>
-      <c r="BF18" s="9"/>
-      <c r="BG18" s="4"/>
+      <c r="BC18" s="9"/>
+      <c r="BD18" s="6"/>
+      <c r="BE18" s="1"/>
+      <c r="BF18" s="6"/>
+      <c r="BG18" s="1"/>
     </row>
-    <row r="19" spans="1:59" ht="7.5" customHeight="1" thickBot="1">
-      <c r="A19" s="12"/>
-      <c r="B19" s="63"/>
-      <c r="C19" s="64"/>
-      <c r="D19" s="65"/>
+    <row r="19" spans="2:59" ht="7.5" customHeight="1" thickBot="1">
+      <c r="B19" s="33"/>
+      <c r="C19" s="34"/>
+      <c r="D19" s="35"/>
       <c r="E19" s="1"/>
-      <c r="F19" s="63"/>
-      <c r="G19" s="64"/>
-      <c r="H19" s="65"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="35"/>
       <c r="I19" s="1"/>
-      <c r="J19" s="75"/>
-      <c r="K19" s="76"/>
-      <c r="L19" s="77"/>
-      <c r="N19" s="81"/>
-      <c r="O19" s="40"/>
-      <c r="P19" s="76"/>
-      <c r="Q19" s="76"/>
-      <c r="R19" s="77"/>
+      <c r="J19" s="56"/>
+      <c r="K19" s="57"/>
+      <c r="L19" s="58"/>
+      <c r="N19" s="59"/>
+      <c r="O19" s="34"/>
+      <c r="P19" s="57"/>
+      <c r="Q19" s="57"/>
+      <c r="R19" s="58"/>
       <c r="S19" s="1"/>
-      <c r="T19" s="94"/>
-      <c r="U19" s="95"/>
-      <c r="V19" s="95"/>
-      <c r="W19" s="95"/>
-      <c r="X19" s="95"/>
-      <c r="Y19" s="95"/>
-      <c r="Z19" s="95"/>
-      <c r="AA19" s="95"/>
-      <c r="AB19" s="95"/>
-      <c r="AC19" s="95"/>
-      <c r="AD19" s="95"/>
-      <c r="AE19" s="95"/>
-      <c r="AF19" s="95"/>
-      <c r="AG19" s="95"/>
-      <c r="AH19" s="95"/>
-      <c r="AI19" s="95"/>
-      <c r="AJ19" s="95"/>
-      <c r="AK19" s="95"/>
-      <c r="AL19" s="96"/>
+      <c r="T19" s="82"/>
+      <c r="U19" s="83"/>
+      <c r="V19" s="83"/>
+      <c r="W19" s="83"/>
+      <c r="X19" s="83"/>
+      <c r="Y19" s="83"/>
+      <c r="Z19" s="83"/>
+      <c r="AA19" s="83"/>
+      <c r="AB19" s="83"/>
+      <c r="AC19" s="83"/>
+      <c r="AD19" s="83"/>
+      <c r="AE19" s="83"/>
+      <c r="AF19" s="83"/>
+      <c r="AG19" s="83"/>
+      <c r="AH19" s="83"/>
+      <c r="AI19" s="83"/>
+      <c r="AJ19" s="83"/>
+      <c r="AK19" s="83"/>
+      <c r="AL19" s="84"/>
       <c r="AM19" s="1"/>
-      <c r="AN19" s="75"/>
-      <c r="AO19" s="76"/>
-      <c r="AP19" s="77"/>
+      <c r="AN19" s="56"/>
+      <c r="AO19" s="57"/>
+      <c r="AP19" s="58"/>
       <c r="AQ19" s="1"/>
-      <c r="AR19" s="75"/>
-      <c r="AS19" s="76"/>
-      <c r="AT19" s="77"/>
+      <c r="AR19" s="56"/>
+      <c r="AS19" s="57"/>
+      <c r="AT19" s="58"/>
       <c r="AU19" s="1"/>
-      <c r="AV19" s="63"/>
-      <c r="AW19" s="64"/>
-      <c r="AX19" s="65"/>
+      <c r="AV19" s="33"/>
+      <c r="AW19" s="34"/>
+      <c r="AX19" s="35"/>
       <c r="AY19" s="1"/>
       <c r="AZ19" s="1"/>
       <c r="BA19" s="1"/>
       <c r="BB19" s="1"/>
       <c r="BC19" s="1"/>
       <c r="BD19" s="1"/>
-      <c r="BE19" s="4"/>
-      <c r="BF19" s="4"/>
-      <c r="BG19" s="4"/>
+      <c r="BE19" s="1"/>
+      <c r="BF19" s="1"/>
+      <c r="BG19" s="1"/>
     </row>
-    <row r="20" spans="1:59" ht="21" thickBot="1">
-      <c r="A20" s="12"/>
-      <c r="B20" s="66" t="s">
+    <row r="20" spans="2:59" ht="22" thickBot="1">
+      <c r="B20" s="73" t="s">
         <v>119</v>
       </c>
-      <c r="C20" s="67"/>
-      <c r="D20" s="68"/>
+      <c r="C20" s="74"/>
+      <c r="D20" s="75"/>
       <c r="E20" s="1"/>
-      <c r="F20" s="66" t="s">
+      <c r="F20" s="73" t="s">
         <v>120</v>
       </c>
-      <c r="G20" s="67"/>
-      <c r="H20" s="68"/>
+      <c r="G20" s="74"/>
+      <c r="H20" s="75"/>
       <c r="I20" s="1"/>
-      <c r="J20" s="78" t="s">
-        <v>132</v>
-      </c>
-      <c r="K20" s="79"/>
-      <c r="L20" s="80"/>
-      <c r="N20" s="66" t="s">
+      <c r="J20" s="76" t="s">
+        <v>131</v>
+      </c>
+      <c r="K20" s="77"/>
+      <c r="L20" s="78"/>
+      <c r="N20" s="73" t="s">
+        <v>128</v>
+      </c>
+      <c r="O20" s="74"/>
+      <c r="P20" s="74"/>
+      <c r="Q20" s="74"/>
+      <c r="R20" s="75"/>
+      <c r="S20" s="1"/>
+      <c r="T20" s="85"/>
+      <c r="U20" s="86"/>
+      <c r="V20" s="86"/>
+      <c r="W20" s="86"/>
+      <c r="X20" s="86"/>
+      <c r="Y20" s="86"/>
+      <c r="Z20" s="86"/>
+      <c r="AA20" s="86"/>
+      <c r="AB20" s="86"/>
+      <c r="AC20" s="86"/>
+      <c r="AD20" s="86"/>
+      <c r="AE20" s="86"/>
+      <c r="AF20" s="86"/>
+      <c r="AG20" s="86"/>
+      <c r="AH20" s="86"/>
+      <c r="AI20" s="86"/>
+      <c r="AJ20" s="86"/>
+      <c r="AK20" s="86"/>
+      <c r="AL20" s="87"/>
+      <c r="AM20" s="1"/>
+      <c r="AN20" s="73" t="s">
+        <v>128</v>
+      </c>
+      <c r="AO20" s="74"/>
+      <c r="AP20" s="75"/>
+      <c r="AQ20" s="1"/>
+      <c r="AR20" s="73" t="s">
         <v>129</v>
       </c>
-      <c r="O20" s="67"/>
-      <c r="P20" s="67"/>
-      <c r="Q20" s="67"/>
-      <c r="R20" s="68"/>
-      <c r="S20" s="1"/>
-      <c r="T20" s="97"/>
-      <c r="U20" s="98"/>
-      <c r="V20" s="98"/>
-      <c r="W20" s="98"/>
-      <c r="X20" s="98"/>
-      <c r="Y20" s="98"/>
-      <c r="Z20" s="98"/>
-      <c r="AA20" s="98"/>
-      <c r="AB20" s="98"/>
-      <c r="AC20" s="98"/>
-      <c r="AD20" s="98"/>
-      <c r="AE20" s="98"/>
-      <c r="AF20" s="98"/>
-      <c r="AG20" s="98"/>
-      <c r="AH20" s="98"/>
-      <c r="AI20" s="98"/>
-      <c r="AJ20" s="98"/>
-      <c r="AK20" s="98"/>
-      <c r="AL20" s="99"/>
-      <c r="AM20" s="1"/>
-      <c r="AN20" s="66" t="s">
-        <v>129</v>
-      </c>
-      <c r="AO20" s="67"/>
-      <c r="AP20" s="68"/>
-      <c r="AQ20" s="1"/>
-      <c r="AR20" s="66" t="s">
-        <v>130</v>
-      </c>
-      <c r="AS20" s="67"/>
-      <c r="AT20" s="68"/>
+      <c r="AS20" s="74"/>
+      <c r="AT20" s="75"/>
       <c r="AU20" s="1"/>
-      <c r="AV20" s="66" t="s">
+      <c r="AV20" s="73" t="s">
         <v>119</v>
       </c>
-      <c r="AW20" s="67"/>
-      <c r="AX20" s="68"/>
+      <c r="AW20" s="74"/>
+      <c r="AX20" s="75"/>
       <c r="AY20" s="1"/>
-      <c r="AZ20" s="89" t="s">
-        <v>140</v>
+      <c r="AZ20" s="66" t="s">
+        <v>139</v>
       </c>
       <c r="BA20" s="1"/>
-      <c r="BB20" s="89" t="s">
-        <v>139</v>
+      <c r="BB20" s="66" t="s">
+        <v>138</v>
       </c>
       <c r="BC20" s="1"/>
-      <c r="BD20" s="89" t="s">
+      <c r="BD20" s="66" t="s">
         <v>106</v>
       </c>
-      <c r="BE20" s="4"/>
-      <c r="BF20" s="9"/>
-      <c r="BG20" s="4"/>
+      <c r="BE20" s="1"/>
+      <c r="BF20" s="6"/>
+      <c r="BG20" s="1"/>
     </row>
-    <row r="21" spans="1:59" ht="4.5" customHeight="1"/>
+    <row r="21" spans="2:59" ht="4.5" customHeight="1"/>
   </sheetData>
   <mergeCells count="14">
     <mergeCell ref="AR18:AT18"/>

</xml_diff>

<commit_message>
Prepare for release 2.1.0
Доработаны раскладки для Windows, для клавиатур ISO клавиша справа от левого шифт @/~.
</commit_message>
<xml_diff>
--- a/Images/WhiskKBLayouts.xlsx
+++ b/Images/WhiskKBLayouts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11008"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/2Data/GitHub/Whiskeroff/WhiskKBLayouts/Images/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/2Data/GitHub/Whiskeroff_3/WhiskKBLayouts/Images/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF31338C-3816-884A-B0A0-B699687B3E5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{113AFA19-3A55-C440-959F-ABED12B8D50F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-33600" yWindow="500" windowWidth="33600" windowHeight="20500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EN&amp;RU by Whisk" sheetId="7" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="142">
   <si>
     <t>&lt;</t>
   </si>
@@ -1546,9 +1546,7 @@
       <c r="AD4" s="27">
         <v>7</v>
       </c>
-      <c r="AE4" s="28">
-        <v>7</v>
-      </c>
+      <c r="AE4" s="28"/>
       <c r="AF4" s="29"/>
       <c r="AG4" s="1"/>
       <c r="AH4" s="27">
@@ -2298,7 +2296,7 @@
       <c r="F14" s="39"/>
       <c r="G14" s="7"/>
       <c r="H14" s="31" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="I14" s="32"/>
       <c r="J14" s="39"/>
@@ -2461,7 +2459,9 @@
       <c r="E16" s="37"/>
       <c r="F16" s="53"/>
       <c r="G16" s="7"/>
-      <c r="H16" s="36"/>
+      <c r="H16" s="36" t="s">
+        <v>6</v>
+      </c>
       <c r="I16" s="37"/>
       <c r="J16" s="53"/>
       <c r="K16" s="7"/>

</xml_diff>